<commit_message>
handling output of non utf8 data over console
</commit_message>
<xml_diff>
--- a/RetailerName.xlsx
+++ b/RetailerName.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cisco-my.sharepoint.com/personal/snardi_cisco_com/Documents/Documents/GitHub/AP_replacement_ph2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="11_2B59D2BFD3605185D4F4D672423088B352998C0D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AC87CE02-67B1-4B26-A62C-CB87E7408F65}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="11_7E1392BA4A10D837413C6E355C484D6F2D2745ED" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CF6DAE3D-FDE0-47D7-B70A-7EDAC1AEBF51}"/>
   <bookViews>
-    <workbookView xWindow="33" yWindow="87" windowWidth="25594" windowHeight="15273" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView minimized="1" xWindow="7" yWindow="727" windowWidth="25593" windowHeight="15273" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -31,9 +31,6 @@
     <t>999999</t>
   </si>
   <si>
-    <t>Test Partner Ltd</t>
-  </si>
-  <si>
     <t>Numeric ID Company</t>
   </si>
   <si>
@@ -41,6 +38,9 @@
   </si>
   <si>
     <t>Another Company</t>
+  </si>
+  <si>
+    <t>ÅÄÖ</t>
   </si>
 </sst>
 </file>
@@ -405,10 +405,6 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B4"/>
   <sheetFormatPr defaultRowHeight="14.35" x14ac:dyDescent="0.5"/>
-  <cols>
-    <col min="1" max="1" width="11.17578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.46875" bestFit="1" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.5">
       <c r="A1" s="1" t="s">
@@ -423,7 +419,7 @@
         <v>2</v>
       </c>
       <c r="B2" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.5">
@@ -431,15 +427,15 @@
         <v>61234</v>
       </c>
       <c r="B3" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.5">
       <c r="A4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" t="s">
         <v>5</v>
-      </c>
-      <c r="B4" t="s">
-        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -449,6 +445,6 @@
 
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
-  <clbl:label id="{c8f49a32-fde3-48a5-9266-b5b0972a22dc}" enabled="1" method="Standard" siteId="{5ae1af62-9505-4097-a69a-c1553ef7840e}" contentBits="2" removed="0"/>
+  <clbl:label id="{c8f49a32-fde3-48a5-9266-b5b0972a22dc}" enabled="1" method="Standard" siteId="{5ae1af62-9505-4097-a69a-c1553ef7840e}" removed="0"/>
 </clbl:labelList>
 </file>
</xml_diff>